<commit_message>
Afegit en SimulacióVenda, la llista de compres afectades per la simulació.
</commit_message>
<xml_diff>
--- a/Docs/SimulacioVenda.xlsx
+++ b/Docs/SimulacioVenda.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319D7ECF-CE53-472E-9801-345361E69E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF696B6-F7BB-496A-A323-2795278C7851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F0182BAC-906E-4536-B8C7-199A601D9A89}"/>
   </bookViews>
   <sheets>
-    <sheet name="Mov 15" sheetId="4" r:id="rId1"/>
-    <sheet name="Deusche" sheetId="1" r:id="rId2"/>
-    <sheet name="Taules" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
+    <sheet name="Mov 15" sheetId="4" r:id="rId2"/>
+    <sheet name="Deusche" sheetId="1" r:id="rId3"/>
+    <sheet name="Taules" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="38">
   <si>
     <t>Data Compra Orig</t>
   </si>
@@ -130,6 +131,24 @@
   </si>
   <si>
     <t>V5</t>
+  </si>
+  <si>
+    <t>Participacions a repartir:</t>
+  </si>
+  <si>
+    <t>Id:</t>
+  </si>
+  <si>
+    <t>Parts Util:</t>
+  </si>
+  <si>
+    <t>IdOrig:</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Correcte</t>
   </si>
 </sst>
 </file>
@@ -555,6 +574,397 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30E2E389-BD5C-425A-AD33-D51EC9058A04}">
+  <dimension ref="B1:G32"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="18.54296875" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.08984375" customWidth="1"/>
+    <col min="6" max="6" width="7.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1">
+        <v>105.53</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2">
+        <v>197</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2">
+        <v>24.54</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3">
+        <v>24.54</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>203</v>
+      </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4">
+        <v>34.723999999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5">
+        <v>29.760999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6">
+        <v>4.9630000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7">
+        <v>205</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7">
+        <v>46.265999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>46.265999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12">
+        <v>197</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12">
+        <v>24.54</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13">
+        <v>24.54</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14">
+        <v>203</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14">
+        <v>34.723999999999997</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15">
+        <v>29.760999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16">
+        <v>37</v>
+      </c>
+      <c r="E16" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16">
+        <v>4.9630000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17">
+        <v>205</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17">
+        <v>0.73599999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18">
+        <v>0.73599999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21">
+        <v>24.54</v>
+      </c>
+      <c r="G21">
+        <f>+F21-F28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22">
+        <v>17</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22">
+        <v>46.265999999999998</v>
+      </c>
+      <c r="G22">
+        <f>+F22-F29</f>
+        <v>45.53</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23">
+        <v>29.760999999999999</v>
+      </c>
+      <c r="G23">
+        <f>+F23-F30</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24">
+        <v>37</v>
+      </c>
+      <c r="E24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24">
+        <v>4.9630000000000001</v>
+      </c>
+      <c r="G24">
+        <f>+F24-F31</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F25" s="1">
+        <f>SUM(F21:F24)</f>
+        <v>105.52999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F27" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28">
+        <v>17</v>
+      </c>
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28">
+        <v>24.54</v>
+      </c>
+      <c r="G28">
+        <f>F21</f>
+        <v>24.54</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29">
+        <v>17</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+      <c r="F29">
+        <v>0.73599999999999999</v>
+      </c>
+      <c r="G29">
+        <v>35.46</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30">
+        <v>29.760999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31">
+        <v>37</v>
+      </c>
+      <c r="E31" t="s">
+        <v>34</v>
+      </c>
+      <c r="F31">
+        <v>4.9630000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F32" s="1">
+        <f>SUM(F28:F31)</f>
+        <v>60</v>
+      </c>
+      <c r="G32">
+        <f>60-SUM(G28:G31)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCF58976-EAE7-4A0A-A776-E4303DC2CBF0}">
   <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1188,7 +1598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8360068-02BA-4318-81EB-89A66DB152B1}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1536,7 +1946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC2FD33C-E4FE-42DC-98BD-EE611A662A9A}">
   <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Mètode compresDeParticions2 utilitzo DesglosCompra en lloc de compra.
</commit_message>
<xml_diff>
--- a/Docs/SimulacioVenda.xlsx
+++ b/Docs/SimulacioVenda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\Meus\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF696B6-F7BB-496A-A323-2795278C7851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{359E9E6A-15FB-41A0-84A8-091921BBC317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F0182BAC-906E-4536-B8C7-199A601D9A89}"/>
   </bookViews>
@@ -215,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -261,6 +261,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,16 +576,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30E2E389-BD5C-425A-AD33-D51EC9058A04}">
-  <dimension ref="B1:G32"/>
+  <dimension ref="B1:I32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="18.54296875" customWidth="1"/>
     <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.08984375" customWidth="1"/>
     <col min="6" max="6" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>32</v>
       </c>
@@ -592,7 +594,7 @@
         <v>105.53</v>
       </c>
     </row>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>33</v>
       </c>
@@ -606,7 +608,7 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>35</v>
       </c>
@@ -620,7 +622,7 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>33</v>
       </c>
@@ -634,7 +636,7 @@
         <v>34.723999999999997</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>35</v>
       </c>
@@ -647,8 +649,11 @@
       <c r="F5">
         <v>29.760999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="I5" s="27">
+        <v>16861.349999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>35</v>
       </c>
@@ -661,8 +666,11 @@
       <c r="F6">
         <v>4.9630000000000001</v>
       </c>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="I6" s="26">
+        <v>4185.07</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>33</v>
       </c>
@@ -675,8 +683,11 @@
       <c r="E7">
         <v>46.265999999999998</v>
       </c>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="I7" s="27">
+        <v>68458.62</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>35</v>
       </c>
@@ -689,8 +700,12 @@
       <c r="F8">
         <v>46.265999999999998</v>
       </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="I8" s="26">
+        <f>SUM(I5:I7)</f>
+        <v>89505.04</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>32</v>
       </c>
@@ -698,7 +713,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>33</v>
       </c>
@@ -712,7 +727,7 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>35</v>
       </c>
@@ -726,7 +741,7 @@
         <v>24.54</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>33</v>
       </c>
@@ -740,7 +755,7 @@
         <v>34.723999999999997</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>35</v>
       </c>
@@ -754,7 +769,7 @@
         <v>29.760999999999999</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>35</v>
       </c>

</xml_diff>